<commit_message>
Actualización automática 2026-09-14 15:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>0</v>
+        <v>214.62</v>
       </c>
       <c r="N7" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>1194.8</v>
+        <v>1836.76</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>3 de 40</t>
+          <t>4 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>1571.02</v>
+        <v>2212.98</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>2602.32</v>
+        <v>3244.28</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>1811.95</v>
+        <v>2668.53</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>35034.05</v>
+        <v>34177.47</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.0491763013624274</v>
+        <v>0.07242387233349618</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>2602.32</v>
+        <v>3458.9</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>44793.31916512035</v>
+        <v>43936.73916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.05490631724437454</v>
+        <v>0.07297928798785971</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-14 17:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1144,10 +1144,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>0</v>
+        <v>1575</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>0</v>
+        <v>87.34999999999999</v>
       </c>
       <c r="J11" s="1" t="n">
         <v>0</v>
@@ -1159,7 +1159,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>0</v>
+        <v>3793.19</v>
       </c>
       <c r="N11" s="1" t="n">
         <v>0</v>
@@ -3005,32 +3005,32 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
+          <t>2 de 40</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>2 de 40</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
           <t>1 de 40</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>1 de 40</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>1 de 40</t>
-        </is>
-      </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>4 de 40</t>
+          <t>5 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3329,7 +3329,7 @@
         <v>84.29000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>0</v>
+        <v>5455.54</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>4000</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>3244.28</v>
+        <v>8699.82</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4216,13 +4216,13 @@
         <v>1339</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>289.8</v>
+        <v>1864.8</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>1049.2</v>
+        <v>-525.8</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.2164301717699776</v>
+        <v>1.392681105302465</v>
       </c>
     </row>
     <row r="8">
@@ -4240,13 +4240,13 @@
         <v>463</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>86.42</v>
+        <v>173.77</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>376.58</v>
+        <v>289.23</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.1866522678185745</v>
+        <v>0.3753131749460044</v>
       </c>
     </row>
     <row r="9">
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>2668.53</v>
+        <v>6461.72</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>34177.47</v>
+        <v>30384.28</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.07242387233349618</v>
+        <v>0.1753710036367584</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>3458.9</v>
+        <v>8914.440000000001</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>43936.73916512034</v>
+        <v>38481.19916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.07297928798785971</v>
+        <v>0.1880856584493614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-15 08:30:20
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -673,13 +673,13 @@
         <v>0</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>0</v>
+        <v>446.68</v>
       </c>
       <c r="L3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>0</v>
+        <v>3213</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>0</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>0</v>
+        <v>337.81</v>
       </c>
       <c r="M11" s="1" t="n">
         <v>3793.19</v>
@@ -3020,17 +3020,17 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>0 de 40</t>
+          <t>1 de 40</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>1 de 40</t>
+          <t>2 de 40</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>5 de 40</t>
+          <t>6 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3167,7 +3167,7 @@
         <v>10.04</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>0</v>
+        <v>3659.68</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>2500</v>
@@ -3329,7 +3329,7 @@
         <v>84.29000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>5455.54</v>
+        <v>5793.35</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>4000</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>8699.82</v>
+        <v>12697.31</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4045,7 +4045,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4312,13 +4312,13 @@
         <v>407.5155</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0</v>
+        <v>446.68</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>407.5155</v>
+        <v>-39.16450000000003</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
+        <v>1.096105546905578</v>
       </c>
     </row>
     <row r="12">
@@ -4360,13 +4360,13 @@
         <v>960</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>337.81</v>
+        <v>675.62</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>622.1900000000001</v>
+        <v>284.38</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.3518854166666667</v>
+        <v>0.7037708333333333</v>
       </c>
     </row>
     <row r="14">
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>6461.72</v>
+        <v>9674.719999999999</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>30384.28</v>
+        <v>27171.28</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.1753710036367584</v>
+        <v>0.2625717852684145</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>8914.440000000001</v>
+        <v>12911.93</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>38481.19916512034</v>
+        <v>34483.70916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.1880856584493614</v>
+        <v>0.2724286501341714</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-15 14:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1399,7 +1399,7 @@
         <v>337.81</v>
       </c>
       <c r="M15" s="1" t="n">
-        <v>0</v>
+        <v>92.88</v>
       </c>
       <c r="N15" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>1836.76</v>
+        <v>2286.86</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>6 de 40</t>
+          <t>7 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3410,7 +3410,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>337.81</v>
+        <v>430.69</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>1500</v>
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>2212.98</v>
+        <v>2663.08</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>12697.31</v>
+        <v>13240.29</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>9674.719999999999</v>
+        <v>10217.7</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>27171.28</v>
+        <v>26628.3</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.2625717852684145</v>
+        <v>0.2773082559843674</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>12911.93</v>
+        <v>13454.91</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>34483.70916512034</v>
+        <v>33940.72916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2724286501341714</v>
+        <v>0.2838849783864042</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-16 14:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>2663.08</v>
+        <v>2701.25</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13240.29</v>
+        <v>13278.46</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4144,13 +4144,13 @@
         <v>3623</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>76.34</v>
+        <v>114.51</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3546.66</v>
+        <v>3508.49</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.02107093568865581</v>
+        <v>0.03160640353298372</v>
       </c>
     </row>
     <row r="5">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>13454.91</v>
+        <v>13493.08</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>33940.72916512034</v>
+        <v>33902.55916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2838849783864042</v>
+        <v>0.2846903267406488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-17 14:30:19
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1399,7 +1399,7 @@
         <v>337.81</v>
       </c>
       <c r="M15" s="1" t="n">
-        <v>92.88</v>
+        <v>105.52</v>
       </c>
       <c r="N15" s="1" t="n">
         <v>0</v>
@@ -3410,7 +3410,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>430.69</v>
+        <v>443.33</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>1500</v>
@@ -3545,7 +3545,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>0</v>
+        <v>38.17</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13278.46</v>
+        <v>13329.27</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4044,7 +4044,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4144,13 +4144,13 @@
         <v>3623</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>114.51</v>
+        <v>152.68</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3508.49</v>
+        <v>3470.32</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.03160640353298372</v>
+        <v>0.04214187137731162</v>
       </c>
     </row>
     <row r="5">
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>10217.7</v>
+        <v>10230.34</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>26628.3</v>
+        <v>26615.66</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.2773082559843674</v>
+        <v>0.2776513054334256</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>13493.08</v>
+        <v>13543.89</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>33902.55916512034</v>
+        <v>33851.74916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2846903267406488</v>
+        <v>0.2857623662973469</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-17 15:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="1" t="n">
-        <v>0</v>
+        <v>2337.66</v>
       </c>
       <c r="N37" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>7 de 40</t>
+          <t>8 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3896,7 +3896,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>0</v>
+        <v>2337.66</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>750</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>13329.27</v>
+        <v>15666.93</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4044,7 +4044,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>10230.34</v>
+        <v>12568</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>26615.66</v>
+        <v>24278</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.2776513054334256</v>
+        <v>0.3410953699180372</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>13543.89</v>
+        <v>15881.55</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>33851.74916512034</v>
+        <v>31514.08916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2857623662973469</v>
+        <v>0.3350846255004751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-17 17:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -3491,7 +3491,7 @@
         <v>23.03</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>429.24</v>
+        <v>431.27</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>1500</v>
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>2701.25</v>
+        <v>2703.28</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15666.93</v>
+        <v>15670.99</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4336,13 +4336,13 @@
         <v>115</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>0</v>
+        <v>4.06</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>115</v>
+        <v>110.94</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0</v>
+        <v>0.03530434782608696</v>
       </c>
     </row>
     <row r="13">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>15881.55</v>
+        <v>15885.61</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>31514.08916512034</v>
+        <v>31510.02916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.3350846255004751</v>
+        <v>0.3351702873898708</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-21 14:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>3213</v>
+        <v>5066.67</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>0</v>
@@ -3167,7 +3167,7 @@
         <v>10.04</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>3659.68</v>
+        <v>5513.35</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>2500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>15670.99</v>
+        <v>17524.66</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4044,7 +4044,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>12568</v>
+        <v>14421.67</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>24278</v>
+        <v>22424.33</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.3410953699180372</v>
+        <v>0.3914039515822613</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>15885.61</v>
+        <v>17739.28</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>31510.02916512034</v>
+        <v>29656.35916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.3351702873898708</v>
+        <v>0.3742808476155078</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-21 15:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -2239,7 +2239,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="1" t="n">
-        <v>0</v>
+        <v>42.48</v>
       </c>
       <c r="N29" s="1" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="1" t="n">
-        <v>2337.66</v>
+        <v>2393.76</v>
       </c>
       <c r="N37" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>8 de 40</t>
+          <t>9 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3734,7 +3734,7 @@
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>0</v>
+        <v>42.48</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>3000</v>
@@ -3896,7 +3896,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>2337.66</v>
+        <v>2393.76</v>
       </c>
       <c r="G30" s="1" t="n">
         <v>750</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>17524.66</v>
+        <v>17623.24</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>14421.67</v>
+        <v>14520.25</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>22424.33</v>
+        <v>22325.75</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.3914039515822613</v>
+        <v>0.3940794116050589</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>17739.28</v>
+        <v>17837.86</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>29656.35916512034</v>
+        <v>29557.77916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.3742808476155078</v>
+        <v>0.376360785806795</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-22 16:30:19
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>2286.86</v>
+        <v>2968.49</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>2703.28</v>
+        <v>3384.91</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>17623.24</v>
+        <v>18304.87</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>14520.25</v>
+        <v>15201.88</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>22325.75</v>
+        <v>21644.12</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.3940794116050589</v>
+        <v>0.4125788416653097</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>17837.86</v>
+        <v>18519.49</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>29557.77916512034</v>
+        <v>28876.14916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.376360785806795</v>
+        <v>0.3907424886808777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-22 17:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1159,7 +1159,7 @@
         <v>337.81</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>3793.19</v>
+        <v>7048.71</v>
       </c>
       <c r="N11" s="1" t="n">
         <v>0</v>
@@ -3329,7 +3329,7 @@
         <v>84.29000000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>5793.35</v>
+        <v>9048.870000000001</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>4000</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>18304.87</v>
+        <v>21560.39</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4044,7 +4044,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>15201.88</v>
+        <v>18457.4</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>21644.12</v>
+        <v>18388.6</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.4125788416653097</v>
+        <v>0.5009336155892092</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>18519.49</v>
+        <v>21775.01</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>28876.14916512034</v>
+        <v>25620.62916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.3907424886808777</v>
+        <v>0.45943066458369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-23 11:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>2968.49</v>
+        <v>3147.34</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>3384.91</v>
+        <v>3563.76</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>21560.39</v>
+        <v>21739.24</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4044,7 +4044,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>18457.4</v>
+        <v>18636.25</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>18388.6</v>
+        <v>18209.75</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5009336155892092</v>
+        <v>0.5057876024534549</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>21775.01</v>
+        <v>21953.86</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>25620.62916512034</v>
+        <v>25441.77916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.45943066458369</v>
+        <v>0.4632042185044823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 14:30:19
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>214.62</v>
+        <v>753.35</v>
       </c>
       <c r="N7" s="1" t="n">
         <v>0</v>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>18636.25</v>
+        <v>19174.98</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>18209.75</v>
+        <v>17671.02</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5057876024534549</v>
+        <v>0.5204087282201596</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>21953.86</v>
+        <v>22492.59</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>25441.77916512034</v>
+        <v>24903.04916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.4632042185044823</v>
+        <v>0.4745708760596876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-29 15:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>3147.34</v>
+        <v>4914.66</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3572,7 +3572,7 @@
         <v>5649.64</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>3563.76</v>
+        <v>5331.08</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>3500</v>
@@ -4021,7 +4021,7 @@
         <v>26526.74</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>21739.24</v>
+        <v>23506.56</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>48710</v>
@@ -4044,7 +4044,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4384,13 +4384,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>19174.98</v>
+        <v>20942.3</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>17671.02</v>
+        <v>15903.7</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5204087282201596</v>
+        <v>0.5683737719155403</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4427,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>22492.59</v>
+        <v>24259.91</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>24903.04916512034</v>
+        <v>23135.72916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.4745708760596876</v>
+        <v>0.5118595387116013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 16:30:19
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CUSTODE FALCONI DIANA CAROLINA</t>
+          <t>CORREA BAUTISTA MONICA ELIZABETH</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
@@ -1219,7 +1219,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="1" t="n">
-        <v>0</v>
+        <v>4289.41</v>
       </c>
       <c r="N12" s="1" t="n">
         <v>0</v>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FLORES MANOSALVAS CHRISTIAN PATRICIO</t>
+          <t>CUSTODE FALCONI DIANA CAROLINA</t>
         </is>
       </c>
       <c r="C13" s="1" t="n">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FREVIUNO CIA. LTDA.</t>
+          <t>FLORES MANOSALVAS CHRISTIAN PATRICIO</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FUENTES PAREDES MARIA FERNANDA</t>
+          <t>FREVIUNO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
@@ -1396,10 +1396,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="1" t="n">
-        <v>337.81</v>
+        <v>0</v>
       </c>
       <c r="M15" s="1" t="n">
-        <v>105.52</v>
+        <v>0</v>
       </c>
       <c r="N15" s="1" t="n">
         <v>0</v>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GARCES VELASCO SOLUAKABADOS CIA.LTDA.</t>
+          <t>FUENTES PAREDES MARIA FERNANDA</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
@@ -1456,10 +1456,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="1" t="n">
-        <v>0</v>
+        <v>337.81</v>
       </c>
       <c r="M16" s="1" t="n">
-        <v>0</v>
+        <v>105.52</v>
       </c>
       <c r="N16" s="1" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GUNSHA MAIGUA SEGUNDO JORGE</t>
+          <t>GARCES VELASCO SOLUAKABADOS CIA.LTDA.</t>
         </is>
       </c>
       <c r="C17" s="1" t="n">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HERRERA CAICEDO LUIS FRANKLIN</t>
+          <t>GUNSHA MAIGUA SEGUNDO JORGE</t>
         </is>
       </c>
       <c r="C18" s="1" t="n">
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>429.24</v>
+        <v>0</v>
       </c>
       <c r="N18" s="1" t="n">
         <v>0</v>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IMPORAKABADOS CIA. LTDA.</t>
+          <t>HERRERA CAICEDO LUIS FRANKLIN</t>
         </is>
       </c>
       <c r="C19" s="1" t="n">
@@ -1639,7 +1639,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="1" t="n">
-        <v>0</v>
+        <v>429.24</v>
       </c>
       <c r="N19" s="1" t="n">
         <v>0</v>
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>INCA VELEZ EDWIN EDGAR</t>
+          <t>IMPORAKABADOS CIA. LTDA.</t>
         </is>
       </c>
       <c r="C20" s="1" t="n">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JAYA TENE MARCO RENE</t>
+          <t>INCA VELEZ EDWIN EDGAR</t>
         </is>
       </c>
       <c r="C21" s="1" t="n">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>LLERENA CONDO SANDRA MARISOL</t>
+          <t>JAYA TENE MARCO RENE</t>
         </is>
       </c>
       <c r="C22" s="1" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MANCHENO PINO HERVIN SANTIAGO</t>
+          <t>LLERENA CONDO SANDRA MARISOL</t>
         </is>
       </c>
       <c r="C23" s="1" t="n">
@@ -1864,10 +1864,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="1" t="n">
-        <v>289.8</v>
+        <v>0</v>
       </c>
       <c r="I23" s="1" t="n">
-        <v>86.42</v>
+        <v>0</v>
       </c>
       <c r="J23" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>4914.66</v>
+        <v>0</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ORTIZ PEREZ KEVIN DAVID</t>
+          <t>MANCHENO PINO HERVIN SANTIAGO</t>
         </is>
       </c>
       <c r="C24" s="1" t="n">
@@ -1924,10 +1924,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>0</v>
+        <v>289.8</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>0</v>
+        <v>86.42</v>
       </c>
       <c r="J24" s="1" t="n">
         <v>0</v>
@@ -1939,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>0</v>
+        <v>4914.66</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>0</v>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OSORIO BASTIDAS FERNANDO JOSELITO</t>
+          <t>ORTIZ PEREZ KEVIN DAVID</t>
         </is>
       </c>
       <c r="C25" s="1" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PALATE CHUCARALAO JOSE ISRAEL</t>
+          <t>OSORIO BASTIDAS FERNANDO JOSELITO</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PEÑAHERRERA MOLINA JORGE OCTAVIO</t>
+          <t>PALATE CHUCARALAO JOSE ISRAEL</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>POLO FUNES DORIS GRACIELA</t>
+          <t>PEÑAHERRERA MOLINA JORGE OCTAVIO</t>
         </is>
       </c>
       <c r="C28" s="1" t="n">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PROVEEDORA PARA METALMECANICA E INDUSTRIAS PROMETIN CIA LTDA</t>
+          <t>POLO FUNES DORIS GRACIELA</t>
         </is>
       </c>
       <c r="C29" s="1" t="n">
@@ -2239,7 +2239,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="1" t="n">
-        <v>42.48</v>
+        <v>0</v>
       </c>
       <c r="N29" s="1" t="n">
         <v>0</v>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>QUINTEROS VELASCO ELSA ROSARIO</t>
+          <t>PROVEEDORA PARA METALMECANICA E INDUSTRIAS PROMETIN CIA LTDA</t>
         </is>
       </c>
       <c r="C30" s="1" t="n">
@@ -2299,7 +2299,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="1" t="n">
-        <v>0</v>
+        <v>42.48</v>
       </c>
       <c r="N30" s="1" t="n">
         <v>0</v>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SANCHEZ BONILLA IGNACIO FERNANDO</t>
+          <t>QUINTEROS VELASCO ELSA ROSARIO</t>
         </is>
       </c>
       <c r="C31" s="1" t="n">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SANCHEZ SARMIENTO ANDRES FERNANDO</t>
+          <t>SANCHEZ BONILLA IGNACIO FERNANDO</t>
         </is>
       </c>
       <c r="C32" s="1" t="n">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SANTANA JIMENEZ MARIA ELENA</t>
+          <t>SANCHEZ SARMIENTO ANDRES FERNANDO</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SILVA GODOY CARMEN TERESA</t>
+          <t>SANTANA JIMENEZ MARIA ELENA</t>
         </is>
       </c>
       <c r="C34" s="1" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SOCIEDAD DE HECHO PROCESA</t>
+          <t>SILVA GODOY CARMEN TERESA</t>
         </is>
       </c>
       <c r="C35" s="1" t="n">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SUAREZ REYES LISBETH JHOMAIRA</t>
+          <t>SOCIEDAD DE HECHO PROCESA</t>
         </is>
       </c>
       <c r="C36" s="1" t="n">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TAMAYO CONDO LUIS ALFREDO</t>
+          <t>SUAREZ REYES LISBETH JHOMAIRA</t>
         </is>
       </c>
       <c r="C37" s="1" t="n">
@@ -2719,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="M37" s="1" t="n">
-        <v>2393.76</v>
+        <v>0</v>
       </c>
       <c r="N37" s="1" t="n">
         <v>0</v>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TIERRA GUAÑO JAIRO GABRIEL</t>
+          <t>TAMAYO CONDO LUIS ALFREDO</t>
         </is>
       </c>
       <c r="C38" s="1" t="n">
@@ -2779,7 +2779,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="1" t="n">
-        <v>0</v>
+        <v>2393.76</v>
       </c>
       <c r="N38" s="1" t="n">
         <v>0</v>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TOAQUIZA VILCA EDISON VLADIMIR</t>
+          <t>TIERRA GUAÑO JAIRO GABRIEL</t>
         </is>
       </c>
       <c r="C39" s="1" t="n">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>VILLAFUERTE MASABANDA JULIO CESAR</t>
+          <t>TOAQUIZA VILCA EDISON VLADIMIR</t>
         </is>
       </c>
       <c r="C40" s="1" t="n">
@@ -2925,137 +2925,197 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>VILLAFUERTE MASABANDA JULIO CESAR</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ALMEIDA CUATIN JHONATHANN CARLOS</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>ZAMBRANO CEDEÑO MARJORIE XIOMARA</t>
         </is>
       </c>
-      <c r="C41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="P41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>2 de 40</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>2 de 40</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>1 de 40</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>2 de 40</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>9 de 40</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="Q42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
-      <c r="R42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
+      <c r="C42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2 de 41</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>2 de 41</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>1 de 41</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>2 de 41</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>10 de 41</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
+        </is>
+      </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>0 de 41</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3343,20 +3403,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CUSTODE FALCONI DIANA CAROLINA</t>
+          <t>CORREA BAUTISTA MONICA ELIZABETH</t>
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>4701.99</v>
+        <v>0</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>3465.88</v>
+        <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>0</v>
+        <v>4289.41</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>0</v>
@@ -3370,23 +3430,23 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FREVIUNO CIA. LTDA.</t>
+          <t>CUSTODE FALCONI DIANA CAROLINA</t>
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>0</v>
+        <v>4701.99</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>0</v>
+        <v>3465.88</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -3397,11 +3457,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FUENTES PAREDES MARIA FERNANDA</t>
+          <t>FREVIUNO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>478.98</v>
+        <v>0</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>0</v>
@@ -3410,10 +3470,10 @@
         <v>0</v>
       </c>
       <c r="F12" s="1" t="n">
-        <v>443.33</v>
+        <v>0</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13">
@@ -3424,23 +3484,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GARCES VELASCO SOLUAKABADOS CIA.LTDA.</t>
+          <t>FUENTES PAREDES MARIA FERNANDA</t>
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>0</v>
+        <v>478.98</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>5918.25</v>
+        <v>0</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>0</v>
+        <v>443.33</v>
       </c>
       <c r="G13" s="1" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="14">
@@ -3451,7 +3511,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GUNSHA MAIGUA SEGUNDO JORGE</t>
+          <t>GARCES VELASCO SOLUAKABADOS CIA.LTDA.</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
@@ -3461,13 +3521,13 @@
         <v>0</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>0</v>
+        <v>5918.25</v>
       </c>
       <c r="F14" s="1" t="n">
-        <v>38.17</v>
+        <v>0</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -3478,23 +3538,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HERRERA CAICEDO LUIS FRANKLIN</t>
+          <t>GUNSHA MAIGUA SEGUNDO JORGE</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>5162.27</v>
+        <v>0</v>
       </c>
       <c r="D15" s="1" t="n">
-        <v>2296.21</v>
+        <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>23.03</v>
+        <v>0</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>431.27</v>
+        <v>38.17</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="16">
@@ -3505,20 +3565,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>INCA VELEZ EDWIN EDGAR</t>
+          <t>HERRERA CAICEDO LUIS FRANKLIN</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>0</v>
+        <v>5162.27</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>0</v>
+        <v>2296.21</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>0</v>
+        <v>23.03</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>0</v>
+        <v>431.27</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>1500</v>
@@ -3532,7 +3592,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LLERENA CONDO SANDRA MARISOL</t>
+          <t>INCA VELEZ EDWIN EDGAR</t>
         </is>
       </c>
       <c r="C17" s="1" t="n">
@@ -3545,10 +3605,10 @@
         <v>0</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>38.17</v>
+        <v>0</v>
       </c>
       <c r="G17" s="1" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="18">
@@ -3559,23 +3619,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MANCHENO PINO HERVIN SANTIAGO</t>
+          <t>LLERENA CONDO SANDRA MARISOL</t>
         </is>
       </c>
       <c r="C18" s="1" t="n">
-        <v>2880.15</v>
+        <v>0</v>
       </c>
       <c r="D18" s="1" t="n">
-        <v>3709.5</v>
+        <v>0</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>5649.64</v>
+        <v>0</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>5331.08</v>
+        <v>38.17</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>3500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
@@ -3586,23 +3646,23 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ORTIZ PEREZ KEVIN DAVID</t>
+          <t>MANCHENO PINO HERVIN SANTIAGO</t>
         </is>
       </c>
       <c r="C19" s="1" t="n">
-        <v>570.5599999999999</v>
+        <v>2880.15</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>6451.27</v>
+        <v>3709.5</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>1133.57</v>
+        <v>5649.64</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>0</v>
+        <v>5331.08</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="20">
@@ -3613,23 +3673,23 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>OSORIO BASTIDAS FERNANDO JOSELITO</t>
+          <t>ORTIZ PEREZ KEVIN DAVID</t>
         </is>
       </c>
       <c r="C20" s="1" t="n">
-        <v>0</v>
+        <v>570.5599999999999</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>0</v>
+        <v>6451.27</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0</v>
+        <v>1133.57</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="1" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="21">
@@ -3640,7 +3700,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PALACIOS CASTRO LUIS SANTIAGO</t>
+          <t>OSORIO BASTIDAS FERNANDO JOSELITO</t>
         </is>
       </c>
       <c r="C21" s="1" t="n">
@@ -3667,14 +3727,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PALATE CHUCARALAO JOSE ISRAEL</t>
+          <t>PALACIOS CASTRO LUIS SANTIAGO</t>
         </is>
       </c>
       <c r="C22" s="1" t="n">
-        <v>99.48</v>
+        <v>0</v>
       </c>
       <c r="D22" s="1" t="n">
-        <v>21.24</v>
+        <v>0</v>
       </c>
       <c r="E22" s="1" t="n">
         <v>0</v>
@@ -3683,7 +3743,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="1" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3694,14 +3754,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>POLO FUNES DORIS GRACIELA</t>
+          <t>PALATE CHUCARALAO JOSE ISRAEL</t>
         </is>
       </c>
       <c r="C23" s="1" t="n">
-        <v>0</v>
+        <v>99.48</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>0</v>
+        <v>21.24</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>0</v>
@@ -3710,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="24">
@@ -3721,23 +3781,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PROVEEDORA PARA METALMECANICA E INDUSTRIAS PROMETIN CIA LTDA</t>
+          <t>POLO FUNES DORIS GRACIELA</t>
         </is>
       </c>
       <c r="C24" s="1" t="n">
-        <v>3858.07</v>
+        <v>0</v>
       </c>
       <c r="D24" s="1" t="n">
-        <v>197.37</v>
+        <v>0</v>
       </c>
       <c r="E24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="1" t="n">
-        <v>42.48</v>
+        <v>0</v>
       </c>
       <c r="G24" s="1" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -3748,23 +3808,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>QUINTEROS VELASCO ELSA ROSARIO</t>
+          <t>PROVEEDORA PARA METALMECANICA E INDUSTRIAS PROMETIN CIA LTDA</t>
         </is>
       </c>
       <c r="C25" s="1" t="n">
-        <v>0</v>
+        <v>3858.07</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>0</v>
+        <v>197.37</v>
       </c>
       <c r="E25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>0</v>
+        <v>42.48</v>
       </c>
       <c r="G25" s="1" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="26">
@@ -3775,14 +3835,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SANCHEZ SARMIENTO ANDRES FERNANDO</t>
+          <t>QUINTEROS VELASCO ELSA ROSARIO</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="1" t="n">
-        <v>2422.57</v>
+        <v>0</v>
       </c>
       <c r="E26" s="1" t="n">
         <v>0</v>
@@ -3791,7 +3851,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
     </row>
     <row r="27">
@@ -3802,14 +3862,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SANTANA JIMENEZ MARIA ELENA</t>
+          <t>SANCHEZ SARMIENTO ANDRES FERNANDO</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>0</v>
+        <v>2422.57</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>0</v>
@@ -3818,7 +3878,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>4560</v>
+        <v>750</v>
       </c>
     </row>
     <row r="28">
@@ -3829,7 +3889,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SILVA GODOY CARMEN TERESA</t>
+          <t>SANTANA JIMENEZ MARIA ELENA</t>
         </is>
       </c>
       <c r="C28" s="1" t="n">
@@ -3845,7 +3905,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>0</v>
+        <v>4560</v>
       </c>
     </row>
     <row r="29">
@@ -3856,14 +3916,14 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SUAREZ REYES LISBETH JHOMAIRA</t>
+          <t>SILVA GODOY CARMEN TERESA</t>
         </is>
       </c>
       <c r="C29" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="1" t="n">
-        <v>1523.9</v>
+        <v>0</v>
       </c>
       <c r="E29" s="1" t="n">
         <v>0</v>
@@ -3883,23 +3943,23 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TAMAYO CONDO LUIS ALFREDO</t>
+          <t>SUAREZ REYES LISBETH JHOMAIRA</t>
         </is>
       </c>
       <c r="C30" s="1" t="n">
-        <v>18.54</v>
+        <v>0</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>0</v>
+        <v>1523.9</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>2393.76</v>
+        <v>0</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>750</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3910,23 +3970,23 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>TIERRA GUAÑO JAIRO GABRIEL</t>
+          <t>TAMAYO CONDO LUIS ALFREDO</t>
         </is>
       </c>
       <c r="C31" s="1" t="n">
-        <v>0</v>
+        <v>18.54</v>
       </c>
       <c r="D31" s="1" t="n">
-        <v>2129.56</v>
+        <v>0</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>2992.49</v>
+        <v>0</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>0</v>
+        <v>2393.76</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>2500</v>
+        <v>750</v>
       </c>
     </row>
     <row r="32">
@@ -3937,23 +3997,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TOAQUIZA VILCA EDISON VLADIMIR</t>
+          <t>TIERRA GUAÑO JAIRO GABRIEL</t>
         </is>
       </c>
       <c r="C32" s="1" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>0</v>
+        <v>2129.56</v>
       </c>
       <c r="E32" s="1" t="n">
-        <v>0</v>
+        <v>2992.49</v>
       </c>
       <c r="F32" s="1" t="n">
         <v>0</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="33">
@@ -3964,7 +4024,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>VILLAFUERTE MASABANDA JULIO CESAR</t>
+          <t>TOAQUIZA VILCA EDISON VLADIMIR</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
@@ -3980,7 +4040,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="34">
@@ -3991,39 +4051,66 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>VILLAFUERTE MASABANDA JULIO CESAR</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ALMEIDA CUATIN JHONATHANN CARLOS</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>ZAMBRANO CEDEÑO MARJORIE XIOMARA</t>
         </is>
       </c>
-      <c r="C34" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="1" t="n">
+      <c r="C35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="1" t="n">
         <v>750</v>
       </c>
     </row>
-    <row r="35">
-      <c r="C35" s="3" t="n">
+    <row r="36">
+      <c r="C36" s="3" t="n">
         <v>28330.07</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D36" s="3" t="n">
         <v>36672.98</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="E36" s="3" t="n">
         <v>26526.74</v>
       </c>
-      <c r="F35" s="3" t="n">
-        <v>23506.56</v>
-      </c>
-      <c r="G35" s="3" t="n">
+      <c r="F36" s="3" t="n">
+        <v>27795.97</v>
+      </c>
+      <c r="G36" s="3" t="n">
         <v>48710</v>
       </c>
     </row>
@@ -4044,7 +4131,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4384,13 +4471,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>20942.3</v>
+        <v>25231.71</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>15903.7</v>
+        <v>11614.29</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5683737719155403</v>
+        <v>0.6847883080931444</v>
       </c>
     </row>
     <row r="15">
@@ -4427,13 +4514,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>24259.91</v>
+        <v>28549.32</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>23135.72916512034</v>
+        <v>18846.31916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.5118595387116013</v>
+        <v>0.6023617468378858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 17:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1219,7 +1219,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="1" t="n">
-        <v>4289.41</v>
+        <v>6355.57</v>
       </c>
       <c r="N12" s="1" t="n">
         <v>0</v>
@@ -1744,7 +1744,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>0</v>
+        <v>1564.2</v>
       </c>
       <c r="I21" s="1" t="n">
         <v>0</v>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>2 de 41</t>
+          <t>3 de 41</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -3416,7 +3416,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>4289.41</v>
+        <v>6355.57</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>0</v>
@@ -3605,7 +3605,7 @@
         <v>0</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>0</v>
+        <v>1564.2</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>1500</v>
@@ -4108,7 +4108,7 @@
         <v>26526.74</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>27795.97</v>
+        <v>31426.33</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48710</v>
@@ -4303,13 +4303,13 @@
         <v>1339</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>1864.8</v>
+        <v>3429</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>-525.8</v>
+        <v>-2090</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>1.392681105302465</v>
+        <v>2.560866318147871</v>
       </c>
     </row>
     <row r="8">
@@ -4471,13 +4471,13 @@
         <v>36846</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>25231.71</v>
+        <v>27297.87</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>11614.29</v>
+        <v>9548.130000000001</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.6847883080931444</v>
+        <v>0.740863865819899</v>
       </c>
     </row>
     <row r="15">
@@ -4514,13 +4514,13 @@
         <v>47395.63916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>28549.32</v>
+        <v>32179.68</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>18846.31916512034</v>
+        <v>15215.95916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.6023617468378858</v>
+        <v>0.6789586672286477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-01 08:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -673,13 +673,13 @@
         <v>0</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>446.68</v>
+        <v>0</v>
       </c>
       <c r="L3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>5066.67</v>
+        <v>0</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>0</v>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>753.35</v>
+        <v>0</v>
       </c>
       <c r="N7" s="1" t="n">
         <v>0</v>
@@ -979,7 +979,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="1" t="n">
-        <v>187.91</v>
+        <v>0</v>
       </c>
       <c r="N8" s="1" t="n">
         <v>0</v>
@@ -1144,10 +1144,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>1575</v>
+        <v>0</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>87.34999999999999</v>
+        <v>0</v>
       </c>
       <c r="J11" s="1" t="n">
         <v>0</v>
@@ -1156,10 +1156,10 @@
         <v>0</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>337.81</v>
+        <v>0</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>7048.71</v>
+        <v>0</v>
       </c>
       <c r="N11" s="1" t="n">
         <v>0</v>
@@ -1219,7 +1219,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="1" t="n">
-        <v>6355.57</v>
+        <v>0</v>
       </c>
       <c r="N12" s="1" t="n">
         <v>0</v>
@@ -1456,10 +1456,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="1" t="n">
-        <v>337.81</v>
+        <v>0</v>
       </c>
       <c r="M16" s="1" t="n">
-        <v>105.52</v>
+        <v>0</v>
       </c>
       <c r="N16" s="1" t="n">
         <v>0</v>
@@ -1639,7 +1639,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="1" t="n">
-        <v>429.24</v>
+        <v>0</v>
       </c>
       <c r="N19" s="1" t="n">
         <v>0</v>
@@ -1744,7 +1744,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="1" t="n">
-        <v>1564.2</v>
+        <v>0</v>
       </c>
       <c r="I21" s="1" t="n">
         <v>0</v>
@@ -1924,10 +1924,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="1" t="n">
-        <v>289.8</v>
+        <v>0</v>
       </c>
       <c r="I24" s="1" t="n">
-        <v>86.42</v>
+        <v>0</v>
       </c>
       <c r="J24" s="1" t="n">
         <v>0</v>
@@ -1939,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>4914.66</v>
+        <v>0</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>0</v>
@@ -2299,7 +2299,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="1" t="n">
-        <v>42.48</v>
+        <v>0</v>
       </c>
       <c r="N30" s="1" t="n">
         <v>0</v>
@@ -2779,7 +2779,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="1" t="n">
-        <v>2393.76</v>
+        <v>0</v>
       </c>
       <c r="N38" s="1" t="n">
         <v>0</v>
@@ -3065,12 +3065,12 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>3 de 41</t>
+          <t>0 de 41</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>2 de 41</t>
+          <t>0 de 41</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3080,17 +3080,17 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>1 de 41</t>
+          <t>0 de 41</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>2 de 41</t>
+          <t>0 de 41</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>10 de 41</t>
+          <t>0 de 41</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3135,10 +3135,10 @@
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3155,22 +3155,22 @@
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>junio</t>
+          <t>julio</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>julio</t>
+          <t>agosto</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>agosto</t>
+          <t>septiembre</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>septiembre</t>
+          <t>octubre</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
@@ -3191,7 +3191,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>26.83</v>
+        <v>0</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>0</v>
@@ -3218,16 +3218,16 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>10129.61</v>
+        <v>1647.96</v>
       </c>
       <c r="D3" s="1" t="n">
-        <v>1647.96</v>
+        <v>10.04</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>10.04</v>
+        <v>5513.35</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>5513.35</v>
+        <v>0</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>2500</v>
@@ -3245,16 +3245,16 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>403.59</v>
+        <v>492.51</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>492.51</v>
+        <v>1163.08</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>1163.08</v>
+        <v>38.17</v>
       </c>
       <c r="F4" s="1" t="n">
-        <v>38.17</v>
+        <v>0</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>1500</v>
@@ -3272,10 +3272,10 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0</v>
+        <v>7922.88</v>
       </c>
       <c r="D5" s="1" t="n">
-        <v>7922.88</v>
+        <v>0</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>0</v>
@@ -3302,13 +3302,13 @@
         <v>0</v>
       </c>
       <c r="D6" s="1" t="n">
-        <v>0</v>
+        <v>775.12</v>
       </c>
       <c r="E6" s="1" t="n">
-        <v>775.12</v>
+        <v>187.91</v>
       </c>
       <c r="F6" s="1" t="n">
-        <v>187.91</v>
+        <v>0</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>2100</v>
@@ -3353,13 +3353,13 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>0</v>
+        <v>4416.81</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>4416.81</v>
+        <v>5311.35</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>5311.35</v>
+        <v>0</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>0</v>
@@ -3380,16 +3380,16 @@
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>0</v>
+        <v>3441.2</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>3441.2</v>
+        <v>84.29000000000001</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>84.29000000000001</v>
+        <v>9048.870000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>9048.870000000001</v>
+        <v>0</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>4000</v>
@@ -3413,10 +3413,10 @@
         <v>0</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>0</v>
+        <v>6355.57</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>6355.57</v>
+        <v>0</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>0</v>
@@ -3434,13 +3434,13 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>4701.99</v>
+        <v>0</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0</v>
+        <v>3465.88</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>3465.88</v>
+        <v>0</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>0</v>
@@ -3488,16 +3488,16 @@
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>478.98</v>
+        <v>0</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>0</v>
+        <v>443.33</v>
       </c>
       <c r="F13" s="1" t="n">
-        <v>443.33</v>
+        <v>0</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>1500</v>
@@ -3518,10 +3518,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>0</v>
+        <v>5918.25</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>5918.25</v>
+        <v>0</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>0</v>
@@ -3548,10 +3548,10 @@
         <v>0</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>0</v>
+        <v>38.17</v>
       </c>
       <c r="F15" s="1" t="n">
-        <v>38.17</v>
+        <v>0</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>500</v>
@@ -3569,16 +3569,16 @@
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>5162.27</v>
+        <v>2296.21</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>2296.21</v>
+        <v>23.03</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>23.03</v>
+        <v>431.27</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>431.27</v>
+        <v>0</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>1500</v>
@@ -3602,10 +3602,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="1" t="n">
-        <v>0</v>
+        <v>1564.2</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>1564.2</v>
+        <v>0</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>1500</v>
@@ -3629,10 +3629,10 @@
         <v>0</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>0</v>
+        <v>38.17</v>
       </c>
       <c r="F18" s="1" t="n">
-        <v>38.17</v>
+        <v>0</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>500</v>
@@ -3650,16 +3650,16 @@
         </is>
       </c>
       <c r="C19" s="1" t="n">
-        <v>2880.15</v>
+        <v>3709.5</v>
       </c>
       <c r="D19" s="1" t="n">
-        <v>3709.5</v>
+        <v>5649.64</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>5649.64</v>
+        <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>5331.08</v>
+        <v>0</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3500</v>
@@ -3677,13 +3677,13 @@
         </is>
       </c>
       <c r="C20" s="1" t="n">
-        <v>570.5599999999999</v>
+        <v>6451.27</v>
       </c>
       <c r="D20" s="1" t="n">
-        <v>6451.27</v>
+        <v>1133.57</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>1133.57</v>
+        <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -3758,10 +3758,10 @@
         </is>
       </c>
       <c r="C23" s="1" t="n">
-        <v>99.48</v>
+        <v>21.24</v>
       </c>
       <c r="D23" s="1" t="n">
-        <v>21.24</v>
+        <v>0</v>
       </c>
       <c r="E23" s="1" t="n">
         <v>0</v>
@@ -3812,16 +3812,16 @@
         </is>
       </c>
       <c r="C25" s="1" t="n">
-        <v>3858.07</v>
+        <v>197.37</v>
       </c>
       <c r="D25" s="1" t="n">
-        <v>197.37</v>
+        <v>0</v>
       </c>
       <c r="E25" s="1" t="n">
-        <v>0</v>
+        <v>42.48</v>
       </c>
       <c r="F25" s="1" t="n">
-        <v>42.48</v>
+        <v>0</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>3000</v>
@@ -3866,10 +3866,10 @@
         </is>
       </c>
       <c r="C27" s="1" t="n">
-        <v>0</v>
+        <v>2422.57</v>
       </c>
       <c r="D27" s="1" t="n">
-        <v>2422.57</v>
+        <v>0</v>
       </c>
       <c r="E27" s="1" t="n">
         <v>0</v>
@@ -3947,10 +3947,10 @@
         </is>
       </c>
       <c r="C30" s="1" t="n">
-        <v>0</v>
+        <v>1523.9</v>
       </c>
       <c r="D30" s="1" t="n">
-        <v>1523.9</v>
+        <v>0</v>
       </c>
       <c r="E30" s="1" t="n">
         <v>0</v>
@@ -3974,16 +3974,16 @@
         </is>
       </c>
       <c r="C31" s="1" t="n">
-        <v>18.54</v>
+        <v>0</v>
       </c>
       <c r="D31" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="1" t="n">
-        <v>0</v>
+        <v>2393.76</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>2393.76</v>
+        <v>0</v>
       </c>
       <c r="G31" s="1" t="n">
         <v>750</v>
@@ -4001,13 +4001,13 @@
         </is>
       </c>
       <c r="C32" s="1" t="n">
-        <v>0</v>
+        <v>2129.56</v>
       </c>
       <c r="D32" s="1" t="n">
-        <v>2129.56</v>
+        <v>2992.49</v>
       </c>
       <c r="E32" s="1" t="n">
-        <v>2992.49</v>
+        <v>0</v>
       </c>
       <c r="F32" s="1" t="n">
         <v>0</v>
@@ -4099,16 +4099,16 @@
     </row>
     <row r="36">
       <c r="C36" s="3" t="n">
-        <v>28330.07</v>
+        <v>36672.98</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>36672.98</v>
+        <v>26526.74</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>26526.74</v>
+        <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>31426.33</v>
+        <v>0</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48710</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-02 15:30:21
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1939,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>0</v>
+        <v>272.94</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>0</v>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>0 de 41</t>
+          <t>1 de 41</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3659,7 +3659,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>0</v>
+        <v>272.94</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>3500</v>
@@ -4108,7 +4108,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>0</v>
+        <v>272.94</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48710</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-06 09:13:45
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -3203,7 +3203,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3">
@@ -3257,7 +3257,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="1" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="5">
@@ -3311,7 +3311,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="1" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
@@ -3338,7 +3338,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="1" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -3365,7 +3365,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="1" t="n">
-        <v>4800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="9">
@@ -3392,7 +3392,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="1" t="n">
-        <v>4000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="10">
@@ -3419,7 +3419,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="1" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="11">
@@ -3446,7 +3446,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="1" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="12">
@@ -3473,7 +3473,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="1" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="13">
@@ -3527,7 +3527,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="1" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="15">
@@ -3554,7 +3554,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="1" t="n">
-        <v>500</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="16">
@@ -3581,7 +3581,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="1" t="n">
-        <v>1500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="17">
@@ -3635,7 +3635,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="1" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="19">
@@ -3662,7 +3662,7 @@
         <v>272.94</v>
       </c>
       <c r="G19" s="1" t="n">
-        <v>3500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="20">
@@ -3770,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="1" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="24">
@@ -3851,7 +3851,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="1" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -3878,7 +3878,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>750</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="28">
@@ -3905,7 +3905,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>4560</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="29">
@@ -3986,7 +3986,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>750</v>
+        <v>500</v>
       </c>
     </row>
     <row r="32">
@@ -4040,7 +4040,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="34">
@@ -4111,7 +4111,7 @@
         <v>272.94</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>48710</v>
+        <v>48250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 08:30:14
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>FLORES MANOSALVAS CHRISTIAN PATRICIO</t>
+          <t>FREVIUNO CIA. LTDA.</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
@@ -1365,7 +1365,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FREVIUNO CIA. LTDA.</t>
+          <t>FUENTES PAREDES MARIA FERNANDA</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FUENTES PAREDES MARIA FERNANDA</t>
+          <t>GARCES VELASCO SOLUAKABADOS CIA.LTDA.</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GARCES VELASCO SOLUAKABADOS CIA.LTDA.</t>
+          <t>GUNSHA MAIGUA SEGUNDO JORGE</t>
         </is>
       </c>
       <c r="C17" s="1" t="n">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GUNSHA MAIGUA SEGUNDO JORGE</t>
+          <t>HERRERA CAICEDO LUIS FRANKLIN</t>
         </is>
       </c>
       <c r="C18" s="1" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HERRERA CAICEDO LUIS FRANKLIN</t>
+          <t>IMPORAKABADOS CIA. LTDA.</t>
         </is>
       </c>
       <c r="C19" s="1" t="n">
@@ -1665,7 +1665,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IMPORAKABADOS CIA. LTDA.</t>
+          <t>INCA VELEZ EDWIN EDGAR</t>
         </is>
       </c>
       <c r="C20" s="1" t="n">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>INCA VELEZ EDWIN EDGAR</t>
+          <t>JAYA TENE MARCO RENE</t>
         </is>
       </c>
       <c r="C21" s="1" t="n">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>JAYA TENE MARCO RENE</t>
+          <t>LLERENA CONDO SANDRA MARISOL</t>
         </is>
       </c>
       <c r="C22" s="1" t="n">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>LLERENA CONDO SANDRA MARISOL</t>
+          <t>MANCHENO PINO HERVIN SANTIAGO</t>
         </is>
       </c>
       <c r="C23" s="1" t="n">
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>0</v>
+        <v>272.94</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MANCHENO PINO HERVIN SANTIAGO</t>
+          <t>ORTIZ PEREZ KEVIN DAVID</t>
         </is>
       </c>
       <c r="C24" s="1" t="n">
@@ -1939,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>272.94</v>
+        <v>0</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>0</v>
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ORTIZ PEREZ KEVIN DAVID</t>
+          <t>OSORIO BASTIDAS FERNANDO JOSELITO</t>
         </is>
       </c>
       <c r="C25" s="1" t="n">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>OSORIO BASTIDAS FERNANDO JOSELITO</t>
+          <t>PALATE CHUCARALAO JOSE ISRAEL</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PALATE CHUCARALAO JOSE ISRAEL</t>
+          <t>PEÑAHERRERA MOLINA JORGE OCTAVIO</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PEÑAHERRERA MOLINA JORGE OCTAVIO</t>
+          <t>POLO FUNES DORIS GRACIELA</t>
         </is>
       </c>
       <c r="C28" s="1" t="n">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>POLO FUNES DORIS GRACIELA</t>
+          <t>PROVEEDORA PARA METALMECANICA E INDUSTRIAS PROMETIN CIA LTDA</t>
         </is>
       </c>
       <c r="C29" s="1" t="n">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PROVEEDORA PARA METALMECANICA E INDUSTRIAS PROMETIN CIA LTDA</t>
+          <t>QUINTEROS VELASCO ELSA ROSARIO</t>
         </is>
       </c>
       <c r="C30" s="1" t="n">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>QUINTEROS VELASCO ELSA ROSARIO</t>
+          <t>SANCHEZ BONILLA IGNACIO FERNANDO</t>
         </is>
       </c>
       <c r="C31" s="1" t="n">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SANCHEZ BONILLA IGNACIO FERNANDO</t>
+          <t>SANCHEZ SARMIENTO ANDRES FERNANDO</t>
         </is>
       </c>
       <c r="C32" s="1" t="n">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SANCHEZ SARMIENTO ANDRES FERNANDO</t>
+          <t>SANTANA JIMENEZ MARIA ELENA</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SANTANA JIMENEZ MARIA ELENA</t>
+          <t>SILVA GODOY CARMEN TERESA</t>
         </is>
       </c>
       <c r="C34" s="1" t="n">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SILVA GODOY CARMEN TERESA</t>
+          <t>SOCIEDAD DE HECHO PROCESA</t>
         </is>
       </c>
       <c r="C35" s="1" t="n">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SOCIEDAD DE HECHO PROCESA</t>
+          <t>SUAREZ REYES LISBETH JHOMAIRA</t>
         </is>
       </c>
       <c r="C36" s="1" t="n">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SUAREZ REYES LISBETH JHOMAIRA</t>
+          <t>TAMAYO CONDO LUIS ALFREDO</t>
         </is>
       </c>
       <c r="C37" s="1" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TAMAYO CONDO LUIS ALFREDO</t>
+          <t>TIERRA GUAÑO JAIRO GABRIEL</t>
         </is>
       </c>
       <c r="C38" s="1" t="n">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIERRA GUAÑO JAIRO GABRIEL</t>
+          <t>TOAQUIZA VILCA EDISON VLADIMIR</t>
         </is>
       </c>
       <c r="C39" s="1" t="n">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TOAQUIZA VILCA EDISON VLADIMIR</t>
+          <t>VILLAFUERTE MASABANDA JULIO CESAR</t>
         </is>
       </c>
       <c r="C40" s="1" t="n">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>VILLAFUERTE MASABANDA JULIO CESAR</t>
+          <t>ZAMBRANO CEDEÑO MARJORIE XIOMARA</t>
         </is>
       </c>
       <c r="C41" s="1" t="n">
@@ -2978,144 +2978,84 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>ALMEIDA CUATIN JHONATHANN CARLOS</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>ZAMBRANO CEDEÑO MARJORIE XIOMARA</t>
-        </is>
-      </c>
-      <c r="C42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="J42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="M42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="N42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="O42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="P42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="L43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>1 de 41</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="O43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="P43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="Q43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
-        </is>
-      </c>
-      <c r="R43" s="2" t="inlineStr">
-        <is>
-          <t>0 de 41</t>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>1 de 40</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>0 de 40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 10:30:14
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>272.94</v>
+        <v>375.29</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>272.94</v>
+        <v>375.29</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>272.94</v>
+        <v>375.29</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 15:30:14
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>0</v>
+        <v>268.27</v>
       </c>
       <c r="N18" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>1 de 40</t>
+          <t>2 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
         <v>431.27</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>0</v>
+        <v>268.27</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>500</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>375.29</v>
+        <v>643.5599999999999</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-08 15:30:15
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>375.29</v>
+        <v>687.98</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>375.29</v>
+        <v>687.98</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>643.5599999999999</v>
+        <v>956.25</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-12 15:30:15
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>687.98</v>
+        <v>873.75</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>687.98</v>
+        <v>873.75</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>956.25</v>
+        <v>1142.02</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 15:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>268.27</v>
+        <v>282.13</v>
       </c>
       <c r="N18" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>873.75</v>
+        <v>1078.45</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3518,7 +3518,7 @@
         <v>431.27</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>268.27</v>
+        <v>282.13</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>500</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>873.75</v>
+        <v>1078.45</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1142.02</v>
+        <v>1360.58</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-13 16:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -4071,8 +4071,8 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4171,13 +4171,13 @@
         <v>3623</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>152.68</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3470.32</v>
+        <v>3623</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.04214187137731162</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -4240,16 +4240,16 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>1339</v>
+        <v>210</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>3429</v>
+        <v>0</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>-2090</v>
+        <v>210</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2.560866318147871</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -4264,16 +4264,16 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>463</v>
+        <v>105</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>173.77</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>289.23</v>
+        <v>105</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.3753131749460044</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4339,13 +4339,13 @@
         <v>407.5155</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>446.68</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>-39.16450000000003</v>
+        <v>407.5155</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>1.096105546905578</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -4363,13 +4363,13 @@
         <v>115</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>4.06</v>
+        <v>0</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>110.94</v>
+        <v>115</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.03530434782608696</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -4387,13 +4387,13 @@
         <v>960</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>675.62</v>
+        <v>0</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>284.38</v>
+        <v>960</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.7037708333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4408,16 +4408,16 @@
         </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>36846</v>
+        <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>27297.87</v>
+        <v>1360.58</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>9548.130000000001</v>
+        <v>37809.53</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.740863865819899</v>
+        <v>0.03473515902814672</v>
       </c>
     </row>
     <row r="15">
@@ -4451,16 +4451,16 @@
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>47395.63916512034</v>
+        <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>32179.68</v>
+        <v>1360.58</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>15215.95916512034</v>
+        <v>46872.16916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.6789586672286477</v>
+        <v>0.02820863466318664</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 10:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>282.13</v>
+        <v>967.71</v>
       </c>
       <c r="N18" s="1" t="n">
         <v>0</v>
@@ -3518,7 +3518,7 @@
         <v>431.27</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>282.13</v>
+        <v>967.71</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>500</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1360.58</v>
+        <v>2046.16</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4073,7 +4073,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>1360.58</v>
+        <v>2046.16</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>37809.53</v>
+        <v>37123.95</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.03473515902814672</v>
+        <v>0.0522377904989289</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>1360.58</v>
+        <v>2046.16</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46872.16916512034</v>
+        <v>46186.58916512033</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.02820863466318664</v>
+        <v>0.0424226285131532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-19 10:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>1078.45</v>
+        <v>1112.57</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>1078.45</v>
+        <v>1112.57</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>2046.16</v>
+        <v>2080.28</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4073,7 +4073,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>2046.16</v>
+        <v>2080.28</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>37123.95</v>
+        <v>37089.83</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.0522377904989289</v>
+        <v>0.05310886285486562</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>2046.16</v>
+        <v>2080.28</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46186.58916512033</v>
+        <v>46152.46916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.0424226285131532</v>
+        <v>0.04313003169025997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-19 16:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -673,13 +673,13 @@
         <v>0</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>0</v>
+        <v>223.34</v>
       </c>
       <c r="L3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>0</v>
+        <v>4024.98</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>0</v>
@@ -1099,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="1" t="n">
-        <v>0</v>
+        <v>186.53</v>
       </c>
       <c r="N10" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>1112.57</v>
+        <v>2030.15</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="P23" s="1" t="n">
-        <v>0</v>
+        <v>1215.33</v>
       </c>
       <c r="Q23" s="1" t="n">
         <v>0</v>
@@ -3020,32 +3020,32 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
+          <t>1 de 40</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
           <t>0 de 40</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>4 de 40</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>0 de 40</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>2 de 40</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr">
+      <c r="O42" s="2" t="inlineStr">
         <is>
           <t>0 de 40</t>
         </is>
       </c>
-      <c r="O42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>0 de 40</t>
+          <t>1 de 40</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
@@ -3167,7 +3167,7 @@
         <v>5513.35</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>0</v>
+        <v>4248.32</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>2500</v>
@@ -3302,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>0</v>
+        <v>186.53</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4000</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>1112.57</v>
+        <v>3245.48</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>2080.28</v>
+        <v>8648.039999999999</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4072,8 +4072,8 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4291,13 +4291,13 @@
         <v>250</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>0</v>
+        <v>1215.33</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>250</v>
+        <v>-965.3299999999999</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0</v>
+        <v>4.86132</v>
       </c>
     </row>
     <row r="10">
@@ -4339,13 +4339,13 @@
         <v>407.5155</v>
       </c>
       <c r="D11" s="1" t="n">
-        <v>0</v>
+        <v>223.34</v>
       </c>
       <c r="E11" s="1" t="n">
-        <v>407.5155</v>
+        <v>184.1755</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0</v>
+        <v>0.5480527734527889</v>
       </c>
     </row>
     <row r="12">
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>2080.28</v>
+        <v>7209.37</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>37089.83</v>
+        <v>31960.74</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.05310886285486562</v>
+        <v>0.1840528402907217</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>2080.28</v>
+        <v>8648.039999999999</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>46152.46916512034</v>
+        <v>39584.70916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.04313003169025997</v>
+        <v>0.1792980941309034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-20 16:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>0</v>
+        <v>851.4400000000001</v>
       </c>
       <c r="N7" s="1" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="P23" s="1" t="n">
-        <v>1215.33</v>
+        <v>1238.7</v>
       </c>
       <c r="Q23" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>4 de 40</t>
+          <t>5 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>3245.48</v>
+        <v>3268.85</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>8648.039999999999</v>
+        <v>8671.41</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4072,7 +4072,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4291,13 +4291,13 @@
         <v>250</v>
       </c>
       <c r="D9" s="1" t="n">
-        <v>1215.33</v>
+        <v>1238.7</v>
       </c>
       <c r="E9" s="1" t="n">
-        <v>-965.3299999999999</v>
+        <v>-988.7</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>4.86132</v>
+        <v>4.954800000000001</v>
       </c>
     </row>
     <row r="10">
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>7209.37</v>
+        <v>8060.81</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>31960.74</v>
+        <v>31109.3</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.1840528402907217</v>
+        <v>0.205789822903229</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>8648.039999999999</v>
+        <v>9522.85</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>39584.70916512034</v>
+        <v>38709.89916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.1792980941309034</v>
+        <v>0.1974353559528487</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-21 14:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1939,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>0</v>
+        <v>655.78</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>5 de 40</t>
+          <t>6 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3626,7 +3626,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>0</v>
+        <v>655.78</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>2500</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>8671.41</v>
+        <v>9327.190000000001</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>8060.81</v>
+        <v>8716.59</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>31109.3</v>
+        <v>30453.52</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.205789822903229</v>
+        <v>0.2225316701944416</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>9522.85</v>
+        <v>10178.63</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>38709.89916512034</v>
+        <v>38054.11916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.1974353559528487</v>
+        <v>0.2110315123269131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 14:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1684,7 +1684,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="1" t="n">
-        <v>0</v>
+        <v>-130.35</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>2030.15</v>
+        <v>2056.98</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -1939,7 +1939,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="1" t="n">
-        <v>655.78</v>
+        <v>792.25</v>
       </c>
       <c r="N24" s="1" t="n">
         <v>0</v>
@@ -3545,7 +3545,7 @@
         <v>1564.2</v>
       </c>
       <c r="F17" s="1" t="n">
-        <v>0</v>
+        <v>-130.35</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>1500</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>3268.85</v>
+        <v>3295.68</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -3626,7 +3626,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="1" t="n">
-        <v>655.78</v>
+        <v>792.25</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>2500</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>9327.190000000001</v>
+        <v>9360.139999999999</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4073,7 +4073,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4243,13 +4243,13 @@
         <v>210</v>
       </c>
       <c r="D7" s="1" t="n">
-        <v>0</v>
+        <v>-130.35</v>
       </c>
       <c r="E7" s="1" t="n">
-        <v>210</v>
+        <v>340.35</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0</v>
+        <v>-0.6207142857142857</v>
       </c>
     </row>
     <row r="8">
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>8716.59</v>
+        <v>8879.889999999999</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>30453.52</v>
+        <v>30290.22</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.2225316701944416</v>
+        <v>0.226700665379801</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>10178.63</v>
+        <v>10211.58</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>38054.11916512034</v>
+        <v>38021.16916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2110315123269131</v>
+        <v>0.2117146581266103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-26 15:30:18
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>2056.98</v>
+        <v>2904.85</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -2779,7 +2779,7 @@
         <v>0</v>
       </c>
       <c r="M38" s="1" t="n">
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="N38" s="1" t="n">
         <v>0</v>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>6 de 40</t>
+          <t>7 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>3295.68</v>
+        <v>4143.55</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -3950,7 +3950,7 @@
         <v>0</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>0</v>
+        <v>40.5</v>
       </c>
       <c r="G32" s="1" t="n">
         <v>2500</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>9360.139999999999</v>
+        <v>10248.51</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>8879.889999999999</v>
+        <v>9768.26</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>30290.22</v>
+        <v>29401.85</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.226700665379801</v>
+        <v>0.2493804587222247</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>10211.58</v>
+        <v>11099.95</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>38021.16916512034</v>
+        <v>37132.79916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2117146581266103</v>
+        <v>0.2301330567328923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-27 14:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1579,7 +1579,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="1" t="n">
-        <v>967.71</v>
+        <v>1008.21</v>
       </c>
       <c r="N18" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>2904.85</v>
+        <v>2958.6</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3518,7 +3518,7 @@
         <v>431.27</v>
       </c>
       <c r="F16" s="1" t="n">
-        <v>967.71</v>
+        <v>1008.21</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>500</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>4143.55</v>
+        <v>4197.3</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>10248.51</v>
+        <v>10342.76</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>9768.26</v>
+        <v>9862.51</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>29401.85</v>
+        <v>29307.6</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.2493804587222247</v>
+        <v>0.2517866301626419</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>11099.95</v>
+        <v>11194.2</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>37132.79916512034</v>
+        <v>37038.54916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2301330567328923</v>
+        <v>0.2320871232464419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-28 15:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>4197.3</v>
+        <v>4652.7</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>10342.76</v>
+        <v>10798.16</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4171,13 +4171,13 @@
         <v>3623</v>
       </c>
       <c r="D4" s="1" t="n">
-        <v>0</v>
+        <v>455.4</v>
       </c>
       <c r="E4" s="1" t="n">
-        <v>3623</v>
+        <v>3167.6</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0</v>
+        <v>0.1256969362406845</v>
       </c>
     </row>
     <row r="5">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>11194.2</v>
+        <v>11649.6</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>37038.54916512034</v>
+        <v>36583.14916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2320871232464419</v>
+        <v>0.2415288409150944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 08:30:16
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1147,7 +1147,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="1" t="n">
-        <v>0</v>
+        <v>480.45</v>
       </c>
       <c r="J11" s="1" t="n">
         <v>0</v>
@@ -1159,7 +1159,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="1" t="n">
-        <v>0</v>
+        <v>2292.78</v>
       </c>
       <c r="N11" s="1" t="n">
         <v>0</v>
@@ -2479,7 +2479,7 @@
         <v>0</v>
       </c>
       <c r="M33" s="1" t="n">
-        <v>0</v>
+        <v>9664.01</v>
       </c>
       <c r="N33" s="1" t="n">
         <v>0</v>
@@ -3010,27 +3010,27 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
+          <t>1 de 40</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
           <t>0 de 40</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>1 de 40</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>0 de 40</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>1 de 40</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>0 de 40</t>
-        </is>
-      </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>7 de 40</t>
+          <t>9 de 40</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3329,7 +3329,7 @@
         <v>9048.870000000001</v>
       </c>
       <c r="F9" s="1" t="n">
-        <v>0</v>
+        <v>2773.23</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>1500</v>
@@ -3842,7 +3842,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>0</v>
+        <v>9664.01</v>
       </c>
       <c r="G28" s="1" t="n">
         <v>3000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>10798.16</v>
+        <v>23235.4</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4267,13 +4267,13 @@
         <v>105</v>
       </c>
       <c r="D8" s="1" t="n">
-        <v>0</v>
+        <v>480.45</v>
       </c>
       <c r="E8" s="1" t="n">
-        <v>105</v>
+        <v>-375.45</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0</v>
+        <v>4.575714285714286</v>
       </c>
     </row>
     <row r="9">
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>9862.51</v>
+        <v>21819.3</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>29307.6</v>
+        <v>17350.81</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.2517866301626419</v>
+        <v>0.5570395385665243</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>11649.6</v>
+        <v>24086.84</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>36583.14916512034</v>
+        <v>24145.90916512035</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2415288409150944</v>
+        <v>0.4993876653711141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 15:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -1099,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="1" t="n">
-        <v>186.53</v>
+        <v>911.46</v>
       </c>
       <c r="N10" s="1" t="n">
         <v>0</v>
@@ -1879,7 +1879,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="1" t="n">
-        <v>2958.6</v>
+        <v>3091.1</v>
       </c>
       <c r="N23" s="1" t="n">
         <v>0</v>
@@ -3302,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="1" t="n">
-        <v>186.53</v>
+        <v>911.46</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>4000</v>
@@ -3599,7 +3599,7 @@
         <v>5331.08</v>
       </c>
       <c r="F19" s="1" t="n">
-        <v>4652.7</v>
+        <v>4785.2</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>4000</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>23235.4</v>
+        <v>24092.83</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4071,7 +4071,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>21819.3</v>
+        <v>22676.73</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>17350.81</v>
+        <v>16493.38</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5570395385665243</v>
+        <v>0.5789294439050592</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>24086.84</v>
+        <v>24944.27</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>24145.90916512035</v>
+        <v>23288.47916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.4993876653711141</v>
+        <v>0.5171645911081205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-30 17:30:17
</commit_message>
<xml_diff>
--- a/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
+++ b/data/ALMEIDA CUATIN JHONATHANN CARLOS.xlsx
@@ -679,7 +679,7 @@
         <v>0</v>
       </c>
       <c r="M3" s="1" t="n">
-        <v>4024.98</v>
+        <v>10062.45</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>0</v>
@@ -919,7 +919,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>851.4400000000001</v>
+        <v>1780.28</v>
       </c>
       <c r="N7" s="1" t="n">
         <v>0</v>
@@ -3078,7 +3078,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -3167,7 +3167,7 @@
         <v>5513.35</v>
       </c>
       <c r="F3" s="1" t="n">
-        <v>4248.32</v>
+        <v>10285.79</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>2500</v>
@@ -4048,7 +4048,7 @@
         <v>31426.33</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>24092.83</v>
+        <v>30130.3</v>
       </c>
       <c r="G36" s="3" t="n">
         <v>48250</v>
@@ -4411,13 +4411,13 @@
         <v>39170.11</v>
       </c>
       <c r="D14" s="1" t="n">
-        <v>22676.73</v>
+        <v>29643.04</v>
       </c>
       <c r="E14" s="1" t="n">
-        <v>16493.38</v>
+        <v>9527.07</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.5789294439050592</v>
+        <v>0.7567770424949024</v>
       </c>
     </row>
     <row r="15">
@@ -4454,13 +4454,13 @@
         <v>48232.74916512034</v>
       </c>
       <c r="D16" s="1" t="n">
-        <v>24944.27</v>
+        <v>31910.58</v>
       </c>
       <c r="E16" s="1" t="n">
-        <v>23288.47916512034</v>
+        <v>16322.16916512034</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.5171645911081205</v>
+        <v>0.6615957114689253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>